<commit_message>
Inclusao de mudanças de layout com CSS
</commit_message>
<xml_diff>
--- a/data/estoque_inicial.xlsx
+++ b/data/estoque_inicial.xlsx
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
     </row>
     <row r="102">
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
     </row>
     <row r="103">

</xml_diff>